<commit_message>
Leave Balance Calculator v2.4 - complete app with data
</commit_message>
<xml_diff>
--- a/Queue_Nature.xlsx
+++ b/Queue_Nature.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="25">
   <si>
     <t xml:space="preserve">Queue</t>
   </si>
@@ -92,6 +92,9 @@
   </si>
   <si>
     <t xml:space="preserve">USMB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WFM</t>
   </si>
 </sst>
 </file>
@@ -106,6 +109,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -178,7 +182,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
@@ -187,15 +191,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -323,7 +327,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -338,7 +342,7 @@
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
     </row>
@@ -346,7 +350,7 @@
       <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>3</v>
       </c>
     </row>
@@ -354,7 +358,7 @@
       <c r="A4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>3</v>
       </c>
     </row>
@@ -362,7 +366,7 @@
       <c r="A5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>3</v>
       </c>
     </row>
@@ -370,7 +374,7 @@
       <c r="A6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>3</v>
       </c>
     </row>
@@ -378,7 +382,7 @@
       <c r="A7" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>3</v>
       </c>
     </row>
@@ -386,7 +390,7 @@
       <c r="A8" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>3</v>
       </c>
     </row>
@@ -394,7 +398,7 @@
       <c r="A9" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>3</v>
       </c>
     </row>
@@ -402,7 +406,7 @@
       <c r="A10" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="1" t="s">
         <v>12</v>
       </c>
     </row>
@@ -410,7 +414,7 @@
       <c r="A11" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="1" t="s">
         <v>12</v>
       </c>
     </row>
@@ -418,7 +422,7 @@
       <c r="A12" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="1" t="s">
         <v>3</v>
       </c>
     </row>
@@ -426,7 +430,7 @@
       <c r="A13" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="1" t="s">
         <v>3</v>
       </c>
     </row>
@@ -434,7 +438,7 @@
       <c r="A14" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="1" t="s">
         <v>12</v>
       </c>
     </row>
@@ -442,7 +446,7 @@
       <c r="A15" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="0" t="s">
+      <c r="B15" s="1" t="s">
         <v>3</v>
       </c>
     </row>
@@ -450,7 +454,7 @@
       <c r="A16" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B16" s="0" t="s">
+      <c r="B16" s="1" t="s">
         <v>3</v>
       </c>
     </row>
@@ -458,7 +462,7 @@
       <c r="A17" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B17" s="0" t="s">
+      <c r="B17" s="1" t="s">
         <v>3</v>
       </c>
     </row>
@@ -466,7 +470,7 @@
       <c r="A18" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B18" s="0" t="s">
+      <c r="B18" s="1" t="s">
         <v>3</v>
       </c>
     </row>
@@ -474,7 +478,7 @@
       <c r="A19" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B19" s="0" t="s">
+      <c r="B19" s="1" t="s">
         <v>3</v>
       </c>
     </row>
@@ -482,7 +486,7 @@
       <c r="A20" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B20" s="0" t="s">
+      <c r="B20" s="1" t="s">
         <v>12</v>
       </c>
     </row>
@@ -490,7 +494,15 @@
       <c r="A21" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B21" s="0" t="s">
+      <c r="B21" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B22" s="1" t="s">
         <v>3</v>
       </c>
     </row>

</xml_diff>